<commit_message>
fix(costs): preserve verified values and improve PDFShift audit
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ops/costs/dcjoineryni-cost-tracker.xlsx
+++ b/ops/costs/dcjoineryni-cost-tracker.xlsx
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -745,12 +745,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hosting plan (Hobby)</t>
+          <t>Database + storage</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -779,17 +779,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Plan detected from Vercel API (28-day audit window).</t>
+          <t>Real amount not inferred. Fill from invoice/export.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Vercel team billing.plan=hobby</t>
+          <t>Credential present, invoice/usage amount still required.</t>
         </is>
       </c>
     </row>
@@ -801,17 +801,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Resend</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Database + storage</t>
+          <t>Transactional email</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
         </is>
       </c>
     </row>
@@ -857,17 +857,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Resend</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Transactional email</t>
+          <t>Model usage</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>AI/API</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
+          <t>status=403 details={'error': "You have insufficient permissions for this operation. Missing scopes: api.usage.read. Check that you have the correct role in your organization, and if you're using a restricted API key, that it has the necessary scopes."}</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Replicate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Model usage</t>
+          <t>Image generation usage</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>status=403 details={'error': "You have insufficient permissions for this operation. Missing scopes: api.usage.read. Check that you have the correct role in your organization, and if you're using a restricted API key, that it has the necessary scopes."}</t>
+          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
         </is>
       </c>
     </row>
@@ -969,17 +969,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Replicate</t>
+          <t>PDFShift</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Image generation usage</t>
+          <t>PDF generation usage</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AI/API</t>
+          <t>Tools</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
+          <t>status=401 mode=basic-fallback details={'success': False, 'error': 'The provided API Key was not found.', 'code': 401}</t>
         </is>
       </c>
     </row>
@@ -1025,22 +1025,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PDFShift</t>
+          <t>Domain Registrar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PDF generation usage</t>
+          <t>dcjoineryni.uk domain</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>yearly</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1059,73 +1059,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Real amount not inferred. Fill from invoice/export.</t>
+          <t>Missing credential/invoice source.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>status=401 details={'success': False, 'error': 'The provided API Key was not found.', 'code': 401}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Domain Registrar</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>dcjoineryni.uk domain</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>yearly</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8">
-        <f>F8*G8</f>
-        <v/>
-      </c>
-      <c r="I8">
-        <f>IF(E8="monthly",H8,IF(E8="yearly",H8/12,0))</f>
-        <v/>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Real amount not inferred. Fill from invoice/export.</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>Missing env key: DOMAIN_INVOICE_REFERENCE</t>
         </is>
       </c>
     </row>
@@ -1925,12 +1869,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Team dc-joinery plan=hobby</t>
+          <t>Team dc-joinery plan=hobby | latest probe: Missing VERCEL_TOKEN for billing audit.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1896,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1918,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1940,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>
@@ -2018,7 +1962,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>
@@ -2035,12 +1979,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>status=401 details={'success': False, 'error': 'The provided API Key was not found.', 'code': 401}</t>
+          <t>status=401 mode=basic-fallback details={'success': False, 'error': 'The provided API Key was not found.', 'code': 401}</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>
@@ -2052,17 +1996,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>Missing env key: DOMAIN_INVOICE_REFERENCE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-22T18:07:20Z</t>
+          <t>2026-07-22T18:09:50Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(costs): refresh tracker artifacts after probe upgrade
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ops/costs/dcjoineryni-cost-tracker.xlsx
+++ b/ops/costs/dcjoineryni-cost-tracker.xlsx
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -745,12 +745,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hosting plan (Hobby)</t>
+          <t>Database + storage</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -779,17 +779,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Plan detected from Vercel API (28-day audit window).</t>
+          <t>Real amount not inferred. Fill from invoice/export.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Vercel team billing.plan=hobby</t>
+          <t>jobs_28d=12 storage_probe_status=406 storage_probe_details={'code': 'PGRST106', 'details': None, 'hint': 'Only the following schemas are exposed: public, graphql_public', 'message': 'Invalid schema: storage'}</t>
         </is>
       </c>
     </row>
@@ -801,17 +801,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Resend</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Database + storage</t>
+          <t>Transactional email</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>emails_28d=0 api_status=200</t>
         </is>
       </c>
     </row>
@@ -857,17 +857,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Resend</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Transactional email</t>
+          <t>Model usage</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>AI/API</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
+          <t>status=403 details={'error': "You have insufficient permissions for this operation. Missing scopes: api.usage.read. Check that you have the correct role in your organization, and if you're using a restricted API key, that it has the necessary scopes."}</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Replicate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Model usage</t>
+          <t>Image generation usage</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>status=403 details={'error': "You have insufficient permissions for this operation. Missing scopes: api.usage.read. Check that you have the correct role in your organization, and if you're using a restricted API key, that it has the necessary scopes."}</t>
+          <t>predictions_28d=5 predict_time_sec_28d=213.86</t>
         </is>
       </c>
     </row>
@@ -969,17 +969,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Replicate</t>
+          <t>PDFShift</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Image generation usage</t>
+          <t>PDF generation usage</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AI/API</t>
+          <t>Tools</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
+          <t>status=401 mode=basic-fallback details={'success': False, 'error': 'The provided API Key was not found.', 'code': 401}</t>
         </is>
       </c>
     </row>
@@ -1025,22 +1025,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PDFShift</t>
+          <t>Domain Registrar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PDF generation usage</t>
+          <t>dcjoineryni.uk domain</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>yearly</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1059,73 +1059,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Real amount not inferred. Fill from invoice/export.</t>
+          <t>Missing credential/invoice source.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>status=401 mode=basic-fallback details={'success': False, 'error': 'The provided API Key was not found.', 'code': 401}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Domain Registrar</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>dcjoineryni.uk domain</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>yearly</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8">
-        <f>F8*G8</f>
-        <v/>
-      </c>
-      <c r="I8">
-        <f>IF(E8="monthly",H8,IF(E8="yearly",H8/12,0))</f>
-        <v/>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Real amount not inferred. Fill from invoice/export.</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>Missing env key: DOMAIN_INVOICE_REFERENCE</t>
         </is>
       </c>
     </row>
@@ -1925,12 +1869,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Team dc-joinery plan=hobby</t>
+          <t>Team dc-joinery plan=hobby | latest probe: Missing VERCEL_TOKEN for billing audit.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>
@@ -1942,17 +1886,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>jobs_28d=12 storage_probe_status=406 storage_probe_details={'code': 'PGRST106', 'details': None, 'hint': 'Only the following schemas are exposed: public, graphql_public', 'message': 'Invalid schema: storage'}</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>
@@ -1964,17 +1908,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
+          <t>emails_28d=0 api_status=200</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1940,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>
@@ -2008,17 +1952,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>status=403 details={'raw': 'error code: 1010\n'}</t>
+          <t>predictions_28d=5 predict_time_sec_28d=213.86</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>
@@ -2040,7 +1984,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>
@@ -2052,17 +1996,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Credential present, invoice/usage amount still required.</t>
+          <t>Missing env key: DOMAIN_INVOICE_REFERENCE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-22T18:10:32Z</t>
+          <t>2026-07-22T18:19:44Z</t>
         </is>
       </c>
     </row>

</xml_diff>